<commit_message>
feat: Add TPM-0515 tarima sync, live github sync button, and email preview image download and clipboard copy buttons
</commit_message>
<xml_diff>
--- a/data/sync_databases/BD_Detalle_Tarimas.xlsx
+++ b/data/sync_databases/BD_Detalle_Tarimas.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H770"/>
+  <dimension ref="A1:H785"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -29680,6 +29680,576 @@
         <v>3</v>
       </c>
     </row>
+    <row r="771">
+      <c r="A771" t="n">
+        <v>815</v>
+      </c>
+      <c r="B771" t="inlineStr">
+        <is>
+          <t>TPM-0515</t>
+        </is>
+      </c>
+      <c r="C771" t="inlineStr">
+        <is>
+          <t>P20512-08</t>
+        </is>
+      </c>
+      <c r="D771" t="inlineStr">
+        <is>
+          <t>URG/GALV</t>
+        </is>
+      </c>
+      <c r="E771" t="inlineStr">
+        <is>
+          <t>INT-047</t>
+        </is>
+      </c>
+      <c r="F771" t="inlineStr">
+        <is>
+          <t>Entrega_P1</t>
+        </is>
+      </c>
+      <c r="G771" t="inlineStr">
+        <is>
+          <t>Proyecto URG/GALV</t>
+        </is>
+      </c>
+      <c r="H771" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="772">
+      <c r="A772" t="n">
+        <v>816</v>
+      </c>
+      <c r="B772" t="inlineStr">
+        <is>
+          <t>TPM-0515</t>
+        </is>
+      </c>
+      <c r="C772" t="inlineStr">
+        <is>
+          <t>P20512-09</t>
+        </is>
+      </c>
+      <c r="D772" t="inlineStr">
+        <is>
+          <t>URG/GALV</t>
+        </is>
+      </c>
+      <c r="E772" t="inlineStr">
+        <is>
+          <t>INT-047</t>
+        </is>
+      </c>
+      <c r="F772" t="inlineStr">
+        <is>
+          <t>Entrega_P1</t>
+        </is>
+      </c>
+      <c r="G772" t="inlineStr">
+        <is>
+          <t>Proyecto URG/GALV</t>
+        </is>
+      </c>
+      <c r="H772" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="773">
+      <c r="A773" t="n">
+        <v>817</v>
+      </c>
+      <c r="B773" t="inlineStr">
+        <is>
+          <t>TPM-0515</t>
+        </is>
+      </c>
+      <c r="C773" t="inlineStr">
+        <is>
+          <t>P17311-17</t>
+        </is>
+      </c>
+      <c r="D773" t="inlineStr">
+        <is>
+          <t>URG/GALV</t>
+        </is>
+      </c>
+      <c r="E773" t="inlineStr">
+        <is>
+          <t>INT-047</t>
+        </is>
+      </c>
+      <c r="F773" t="inlineStr">
+        <is>
+          <t>Entrega_P1</t>
+        </is>
+      </c>
+      <c r="G773" t="inlineStr">
+        <is>
+          <t>Proyecto URG/GALV</t>
+        </is>
+      </c>
+      <c r="H773" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="774">
+      <c r="A774" t="n">
+        <v>818</v>
+      </c>
+      <c r="B774" t="inlineStr">
+        <is>
+          <t>TPM-0515</t>
+        </is>
+      </c>
+      <c r="C774" t="inlineStr">
+        <is>
+          <t>P20153S-04</t>
+        </is>
+      </c>
+      <c r="D774" t="inlineStr">
+        <is>
+          <t>URG/GALV</t>
+        </is>
+      </c>
+      <c r="E774" t="inlineStr">
+        <is>
+          <t>INT-047</t>
+        </is>
+      </c>
+      <c r="F774" t="inlineStr">
+        <is>
+          <t>Entrega_P1</t>
+        </is>
+      </c>
+      <c r="G774" t="inlineStr">
+        <is>
+          <t>Proyecto URG/GALV</t>
+        </is>
+      </c>
+      <c r="H774" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="775">
+      <c r="A775" t="n">
+        <v>819</v>
+      </c>
+      <c r="B775" t="inlineStr">
+        <is>
+          <t>TPM-0515</t>
+        </is>
+      </c>
+      <c r="C775" t="inlineStr">
+        <is>
+          <t>P20321S-05</t>
+        </is>
+      </c>
+      <c r="D775" t="inlineStr">
+        <is>
+          <t>URG/GALV</t>
+        </is>
+      </c>
+      <c r="E775" t="inlineStr">
+        <is>
+          <t>INT-047</t>
+        </is>
+      </c>
+      <c r="F775" t="inlineStr">
+        <is>
+          <t>Entrega_P1</t>
+        </is>
+      </c>
+      <c r="G775" t="inlineStr">
+        <is>
+          <t>Proyecto URG/GALV</t>
+        </is>
+      </c>
+      <c r="H775" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="776">
+      <c r="A776" t="n">
+        <v>820</v>
+      </c>
+      <c r="B776" t="inlineStr">
+        <is>
+          <t>TPM-0515</t>
+        </is>
+      </c>
+      <c r="C776" t="inlineStr">
+        <is>
+          <t>P20321S-06</t>
+        </is>
+      </c>
+      <c r="D776" t="inlineStr">
+        <is>
+          <t>URG/GALV</t>
+        </is>
+      </c>
+      <c r="E776" t="inlineStr">
+        <is>
+          <t>INT-047</t>
+        </is>
+      </c>
+      <c r="F776" t="inlineStr">
+        <is>
+          <t>Entrega_P1</t>
+        </is>
+      </c>
+      <c r="G776" t="inlineStr">
+        <is>
+          <t>Proyecto URG/GALV</t>
+        </is>
+      </c>
+      <c r="H776" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="777">
+      <c r="A777" t="n">
+        <v>821</v>
+      </c>
+      <c r="B777" t="inlineStr">
+        <is>
+          <t>TPM-0515</t>
+        </is>
+      </c>
+      <c r="C777" t="inlineStr">
+        <is>
+          <t>12-6383-01</t>
+        </is>
+      </c>
+      <c r="D777" t="inlineStr">
+        <is>
+          <t>URG/GALV</t>
+        </is>
+      </c>
+      <c r="E777" t="inlineStr">
+        <is>
+          <t>INT-047</t>
+        </is>
+      </c>
+      <c r="F777" t="inlineStr">
+        <is>
+          <t>Entrega_P1</t>
+        </is>
+      </c>
+      <c r="G777" t="inlineStr">
+        <is>
+          <t>Proyecto URG/GALV</t>
+        </is>
+      </c>
+      <c r="H777" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="778">
+      <c r="A778" t="n">
+        <v>822</v>
+      </c>
+      <c r="B778" t="inlineStr">
+        <is>
+          <t>TPM-0515</t>
+        </is>
+      </c>
+      <c r="C778" t="inlineStr">
+        <is>
+          <t>PP20204-12</t>
+        </is>
+      </c>
+      <c r="D778" t="inlineStr">
+        <is>
+          <t>URG/GALV</t>
+        </is>
+      </c>
+      <c r="E778" t="inlineStr">
+        <is>
+          <t>INT-047</t>
+        </is>
+      </c>
+      <c r="F778" t="inlineStr">
+        <is>
+          <t>Entrega_P1</t>
+        </is>
+      </c>
+      <c r="G778" t="inlineStr">
+        <is>
+          <t>Proyecto URG/GALV</t>
+        </is>
+      </c>
+      <c r="H778" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="779">
+      <c r="A779" t="n">
+        <v>823</v>
+      </c>
+      <c r="B779" t="inlineStr">
+        <is>
+          <t>TPM-0515</t>
+        </is>
+      </c>
+      <c r="C779" t="inlineStr">
+        <is>
+          <t>PP20203-13</t>
+        </is>
+      </c>
+      <c r="D779" t="inlineStr">
+        <is>
+          <t>URG/GALV</t>
+        </is>
+      </c>
+      <c r="E779" t="inlineStr">
+        <is>
+          <t>INT-047</t>
+        </is>
+      </c>
+      <c r="F779" t="inlineStr">
+        <is>
+          <t>Entrega_P1</t>
+        </is>
+      </c>
+      <c r="G779" t="inlineStr">
+        <is>
+          <t>Proyecto URG/GALV</t>
+        </is>
+      </c>
+      <c r="H779" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="780">
+      <c r="A780" t="n">
+        <v>824</v>
+      </c>
+      <c r="B780" t="inlineStr">
+        <is>
+          <t>TPM-0515</t>
+        </is>
+      </c>
+      <c r="C780" t="inlineStr">
+        <is>
+          <t>12-6267-01</t>
+        </is>
+      </c>
+      <c r="D780" t="inlineStr">
+        <is>
+          <t>URG/GALV</t>
+        </is>
+      </c>
+      <c r="E780" t="inlineStr">
+        <is>
+          <t>INT-047</t>
+        </is>
+      </c>
+      <c r="F780" t="inlineStr">
+        <is>
+          <t>Entrega_P1</t>
+        </is>
+      </c>
+      <c r="G780" t="inlineStr">
+        <is>
+          <t>Proyecto URG/GALV</t>
+        </is>
+      </c>
+      <c r="H780" t="n">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="781">
+      <c r="A781" t="n">
+        <v>825</v>
+      </c>
+      <c r="B781" t="inlineStr">
+        <is>
+          <t>TPM-0515</t>
+        </is>
+      </c>
+      <c r="C781" t="inlineStr">
+        <is>
+          <t>96-6183-02</t>
+        </is>
+      </c>
+      <c r="D781" t="inlineStr">
+        <is>
+          <t>URG/GALV</t>
+        </is>
+      </c>
+      <c r="E781" t="inlineStr">
+        <is>
+          <t>INT-047</t>
+        </is>
+      </c>
+      <c r="F781" t="inlineStr">
+        <is>
+          <t>Entrega_P1</t>
+        </is>
+      </c>
+      <c r="G781" t="inlineStr">
+        <is>
+          <t>Proyecto URG/GALV</t>
+        </is>
+      </c>
+      <c r="H781" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="782">
+      <c r="A782" t="n">
+        <v>826</v>
+      </c>
+      <c r="B782" t="inlineStr">
+        <is>
+          <t>TPM-0515</t>
+        </is>
+      </c>
+      <c r="C782" t="inlineStr">
+        <is>
+          <t>12-6265-01</t>
+        </is>
+      </c>
+      <c r="D782" t="inlineStr">
+        <is>
+          <t>URG/GALV</t>
+        </is>
+      </c>
+      <c r="E782" t="inlineStr">
+        <is>
+          <t>INT-047</t>
+        </is>
+      </c>
+      <c r="F782" t="inlineStr">
+        <is>
+          <t>Entrega_P1</t>
+        </is>
+      </c>
+      <c r="G782" t="inlineStr">
+        <is>
+          <t>Proyecto URG/GALV</t>
+        </is>
+      </c>
+      <c r="H782" t="n">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="783">
+      <c r="A783" t="n">
+        <v>827</v>
+      </c>
+      <c r="B783" t="inlineStr">
+        <is>
+          <t>TPM-0515</t>
+        </is>
+      </c>
+      <c r="C783" t="inlineStr">
+        <is>
+          <t>11-A-6030-01</t>
+        </is>
+      </c>
+      <c r="D783" t="inlineStr">
+        <is>
+          <t>URG/GALV</t>
+        </is>
+      </c>
+      <c r="E783" t="inlineStr">
+        <is>
+          <t>INT-047</t>
+        </is>
+      </c>
+      <c r="F783" t="inlineStr">
+        <is>
+          <t>Entrega_P1</t>
+        </is>
+      </c>
+      <c r="G783" t="inlineStr">
+        <is>
+          <t>Proyecto URG/GALV</t>
+        </is>
+      </c>
+      <c r="H783" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="784">
+      <c r="A784" t="n">
+        <v>828</v>
+      </c>
+      <c r="B784" t="inlineStr">
+        <is>
+          <t>TPM-0515</t>
+        </is>
+      </c>
+      <c r="C784" t="inlineStr">
+        <is>
+          <t>11-A-6037-01</t>
+        </is>
+      </c>
+      <c r="D784" t="inlineStr">
+        <is>
+          <t>URG/GALV</t>
+        </is>
+      </c>
+      <c r="E784" t="inlineStr">
+        <is>
+          <t>INT-047</t>
+        </is>
+      </c>
+      <c r="F784" t="inlineStr">
+        <is>
+          <t>Entrega_P1</t>
+        </is>
+      </c>
+      <c r="G784" t="inlineStr">
+        <is>
+          <t>Proyecto URG/GALV</t>
+        </is>
+      </c>
+      <c r="H784" t="n">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="785">
+      <c r="A785" t="n">
+        <v>829</v>
+      </c>
+      <c r="B785" t="inlineStr">
+        <is>
+          <t>TPM-0515</t>
+        </is>
+      </c>
+      <c r="C785" t="inlineStr">
+        <is>
+          <t>11-D-6165-01</t>
+        </is>
+      </c>
+      <c r="D785" t="inlineStr">
+        <is>
+          <t>URG/GALV</t>
+        </is>
+      </c>
+      <c r="E785" t="inlineStr">
+        <is>
+          <t>INT-047</t>
+        </is>
+      </c>
+      <c r="F785" t="inlineStr">
+        <is>
+          <t>Entrega_P1</t>
+        </is>
+      </c>
+      <c r="G785" t="inlineStr">
+        <is>
+          <t>Proyecto URG/GALV</t>
+        </is>
+      </c>
+      <c r="H785" t="n">
+        <v>68</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>